<commit_message>
feat: complete leads recap enhancements - referral, ach logic, dashboard sync, and role access
</commit_message>
<xml_diff>
--- a/Data Siswa/Salma.xlsx
+++ b/Data Siswa/Salma.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rupa-Rupa\DashboardTim\Data Siswa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA3942B-C4E5-4343-A442-77B47801BCBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2093E7F8-CB98-4CA4-939D-3E0552E7CB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AFE1E578-4FF8-4474-9732-22FF9E651C93}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="257">
   <si>
     <t>Nama Siswa</t>
   </si>
@@ -804,6 +804,9 @@
   </si>
   <si>
     <t>MOH.AFRIAN</t>
+  </si>
+  <si>
+    <t>SALMA1</t>
   </si>
 </sst>
 </file>
@@ -1372,7 +1375,7 @@
         <v>146</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.35">
@@ -1452,7 +1455,7 @@
         <v>146</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.35">
@@ -1472,7 +1475,7 @@
         <v>146</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.35">
@@ -1492,7 +1495,7 @@
         <v>146</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.35">
@@ -1572,7 +1575,7 @@
         <v>146</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.35">

</xml_diff>